<commit_message>
Hoàn thiện tính năng và cập nhật README
</commit_message>
<xml_diff>
--- a/docs/Estimation-WBS.xlsx
+++ b/docs/Estimation-WBS.xlsx
@@ -11,7 +11,7 @@
     <sheet name="WBS Estimation" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'WBS Estimation'!$A$1:$E$55</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'WBS Estimation'!$A$1:$E$68</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,15 +23,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
   <si>
     <t xml:space="preserve">BẢNG ƯỚC LƯỢNG THỜI GIAN (WORK BREAKDOWN STRUCTURE)</t>
   </si>
   <si>
-    <t xml:space="preserve">Mini Customer Management System — Phase 1 Estimation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đơn vị: giờ công (h)  ·  1 ngày làm việc = 8 giờ  ·  Ngày lập: 15/09/2026</t>
+    <t xml:space="preserve">Mini Customer Management System — Phase 1 Estimation (bổ sung phạm vi phát sinh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đơn vị: giờ công (h)  ·  1 ngày làm việc = 8 giờ  ·  Ngày lập: 15/09/2026  ·  Cập nhật: 17/09/2026</t>
   </si>
   <si>
     <t xml:space="preserve">STT</t>
@@ -259,7 +259,70 @@
     <t xml:space="preserve">Tổng 9. Xử lý Concurrency &amp; Hoàn thiện</t>
   </si>
   <si>
+    <t xml:space="preserve">10. Mở rộng sau MVP (phát sinh 16/09/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sửa lỗi khởi động API (cấu hình Output Cache/Redis) và lỗi JWT không gắn header (DI scope của TokenProvider)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit 921ecf6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thêm EFCore.Design, sinh migration InitialCreate; cấu hình F5/tasks cho VS Code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit 921ecf6, ace7640</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theme nhận diện CEP (AppTheme), dark mode (ThemeService), MainLayout sidebar + AppBar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit 5faa600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trang Dashboard KPI (/) và trang Chi tiết khách hàng (/customers/{id})</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số liệu thật từ API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nâng cấp CustomerList (Filter Drawer, xóa hàng loạt, card view mobile), Command Palette Ctrl+K, làm lại trang Login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AuditLog: entity, AuditLogInterceptor (Old/New JSON), migration AddAuditLogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit 1005bcc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API GET /api/customers/{id}/audit-logs + UI "Lịch sử thay đổi" + 4 unit test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refresh token (chỉ lưu SHA-256 hash, rotation), API refresh/logout, SilentRefreshScheduler phía Blazor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit dde5066</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account lockout (5 lần sai / khóa 15 phút, trả 423) + migration AddRefreshTokenAndLockout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security headers, HSTS, ẩn Server header, thu hẹp CORS; cập nhật AuthServiceTests (34 test)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cập nhật tài liệu: README, ghi chú quyết định bảo mật, Postman, Demo script, Word/Excel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit 732cb1f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tổng 10. Mở rộng sau MVP (phát sinh 16/09/2026)</t>
+  </si>
+  <si>
     <t xml:space="preserve">TỔNG CỘNG TOÀN DỰ ÁN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ghi chú: nhóm 1–9 giữ nguyên ước lượng gốc lập ngày 15/09/2026 (46.0h). Nhóm 10 là ước lượng bổ sung cho phạm vi phát sinh sau MVP, quy đổi từ các commit ngày 16/09/2026.</t>
   </si>
 </sst>
 </file>
@@ -436,11 +499,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -507,6 +574,10 @@
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -761,732 +832,912 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="34"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="25.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="6" t="s">
+    <row r="6" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="D6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="n">
+    <row r="7" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="9" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="E7" s="10"/>
-    </row>
-    <row r="8" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
+      <c r="E7" s="11"/>
+    </row>
+    <row r="8" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="7"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="n">
+      <c r="D8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="9" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="10"/>
+      <c r="D9" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="12" t="n">
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="13" t="n">
         <f aca="false">SUM(D6:D9)</f>
         <v>3.5</v>
       </c>
-      <c r="E10" s="13"/>
+      <c r="E10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="9" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="10" t="s">
+      <c r="D12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="7"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
+      <c r="D13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="8"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="9" t="s">
+      <c r="B14" s="7"/>
+      <c r="C14" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="10" t="s">
+      <c r="D14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6" t="s">
+      <c r="B15" s="7"/>
+      <c r="C15" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="7" t="s">
+      <c r="D15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="12" t="n">
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="13" t="n">
         <f aca="false">SUM(D11:D15)</f>
         <v>4.5</v>
       </c>
-      <c r="E16" s="13"/>
-    </row>
-    <row r="17" customFormat="false" ht="25.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="n">
+      <c r="E16" s="14"/>
+    </row>
+    <row r="17" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="D17" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="E17" s="10"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="n">
+      <c r="E17" s="11"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="6" t="s">
+      <c r="B18" s="10"/>
+      <c r="C18" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="7" t="s">
+      <c r="D18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="n">
+    <row r="19" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9" t="s">
+      <c r="B19" s="10"/>
+      <c r="C19" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="D19" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="10"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="n">
+      <c r="E19" s="11"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="6" t="s">
+      <c r="B20" s="10"/>
+      <c r="C20" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="5" t="n">
+      <c r="D20" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="E20" s="7"/>
+      <c r="E20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="12" t="n">
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="13" t="n">
         <f aca="false">SUM(D17:D20)</f>
         <v>6</v>
       </c>
-      <c r="E21" s="13"/>
+      <c r="E21" s="14"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="n">
+      <c r="A22" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D22" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="E22" s="10"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="n">
+      <c r="E22" s="11"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="6" t="s">
+      <c r="B23" s="10"/>
+      <c r="C23" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D23" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="7"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="n">
+      <c r="D23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9" t="s">
+      <c r="B24" s="10"/>
+      <c r="C24" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="10"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="n">
+      <c r="D24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="11"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="6" t="s">
+      <c r="B25" s="10"/>
+      <c r="C25" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D25" s="5" t="n">
+      <c r="D25" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="E25" s="7"/>
+      <c r="E25" s="8"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="12" t="n">
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="13" t="n">
         <f aca="false">SUM(D22:D25)</f>
         <v>4</v>
       </c>
-      <c r="E26" s="13"/>
+      <c r="E26" s="14"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="n">
+      <c r="A27" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="D27" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="10" t="s">
+      <c r="D27" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="6" t="s">
+      <c r="B28" s="10"/>
+      <c r="C28" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D28" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="7"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="n">
+      <c r="D28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="8"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9" t="s">
+      <c r="B29" s="10"/>
+      <c r="C29" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D29" s="8" t="n">
+      <c r="D29" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E29" s="11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B30" s="9"/>
-      <c r="C30" s="6" t="s">
+      <c r="B30" s="10"/>
+      <c r="C30" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D30" s="5" t="n">
+      <c r="D30" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="8" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9" t="s">
+      <c r="B31" s="10"/>
+      <c r="C31" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D31" s="8" t="n">
+      <c r="D31" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E31" s="11" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B32" s="9"/>
-      <c r="C32" s="6" t="s">
+      <c r="B32" s="10"/>
+      <c r="C32" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="D32" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" s="7" t="s">
+      <c r="D32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="8" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="12" t="n">
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="13" t="n">
         <f aca="false">SUM(D27:D32)</f>
         <v>7.5</v>
       </c>
-      <c r="E33" s="13"/>
+      <c r="E33" s="14"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="8" t="n">
+      <c r="A34" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D34" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="10"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="n">
+      <c r="D34" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="11"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B35" s="9"/>
-      <c r="C35" s="6" t="s">
+      <c r="B35" s="10"/>
+      <c r="C35" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D35" s="5" t="n">
+      <c r="D35" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="E35" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="8" t="n">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9" t="s">
+      <c r="B36" s="10"/>
+      <c r="C36" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="D36" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="10"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="n">
+      <c r="D36" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="11"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B37" s="9"/>
-      <c r="C37" s="6" t="s">
+      <c r="B37" s="10"/>
+      <c r="C37" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="D37" s="5" t="n">
+      <c r="D37" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="E37" s="7"/>
+      <c r="E37" s="8"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11" t="s">
+      <c r="A38" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B38" s="11"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="12" t="n">
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="13" t="n">
         <f aca="false">SUM(D34:D37)</f>
         <v>5</v>
       </c>
-      <c r="E38" s="13"/>
+      <c r="E38" s="14"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="8" t="n">
+      <c r="A39" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="B39" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="D39" s="8" t="n">
+      <c r="D39" s="9" t="n">
         <v>2.5</v>
       </c>
-      <c r="E39" s="10" t="s">
+      <c r="E39" s="11" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="n">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B40" s="9"/>
-      <c r="C40" s="6" t="s">
+      <c r="B40" s="10"/>
+      <c r="C40" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="D40" s="5" t="n">
+      <c r="D40" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="E40" s="7"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="8" t="n">
+      <c r="E40" s="8"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B41" s="9"/>
-      <c r="C41" s="9" t="s">
+      <c r="B41" s="10"/>
+      <c r="C41" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D41" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" s="10"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="n">
+      <c r="D41" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="11"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="B42" s="9"/>
-      <c r="C42" s="6" t="s">
+      <c r="B42" s="10"/>
+      <c r="C42" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" s="7"/>
+      <c r="D42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="8"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="11" t="s">
+      <c r="A43" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="B43" s="11"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="12" t="n">
+      <c r="B43" s="12"/>
+      <c r="C43" s="12"/>
+      <c r="D43" s="13" t="n">
         <f aca="false">SUM(D39:D42)</f>
         <v>6</v>
       </c>
-      <c r="E43" s="13"/>
+      <c r="E43" s="14"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="8" t="n">
+      <c r="A44" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="B44" s="9" t="s">
+      <c r="B44" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D44" s="8" t="n">
+      <c r="D44" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E44" s="10"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="n">
+      <c r="E44" s="11"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="B45" s="9"/>
-      <c r="C45" s="6" t="s">
+      <c r="B45" s="10"/>
+      <c r="C45" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D45" s="5" t="n">
+      <c r="D45" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="E45" s="7"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="8" t="n">
+      <c r="E45" s="8"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9" t="s">
+      <c r="B46" s="10"/>
+      <c r="C46" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="D46" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" s="10"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="n">
+      <c r="D46" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="11"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="B47" s="9"/>
-      <c r="C47" s="6" t="s">
+      <c r="B47" s="10"/>
+      <c r="C47" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D47" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="7"/>
+      <c r="D47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="8"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="11" t="s">
+      <c r="A48" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B48" s="11"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="12" t="n">
+      <c r="B48" s="12"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="13" t="n">
         <f aca="false">SUM(D44:D47)</f>
         <v>5.5</v>
       </c>
-      <c r="E48" s="13"/>
+      <c r="E48" s="14"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="8" t="n">
+      <c r="A49" s="9" t="n">
         <v>36</v>
       </c>
-      <c r="B49" s="9" t="s">
+      <c r="B49" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="D49" s="8" t="n">
+      <c r="D49" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="E49" s="10"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="n">
+      <c r="E49" s="11"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="B50" s="9"/>
-      <c r="C50" s="6" t="s">
+      <c r="B50" s="10"/>
+      <c r="C50" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D50" s="5" t="n">
+      <c r="D50" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="E50" s="7" t="s">
+      <c r="E50" s="8" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="8" t="n">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="9" t="n">
         <v>38</v>
       </c>
-      <c r="B51" s="9"/>
-      <c r="C51" s="9" t="s">
+      <c r="B51" s="10"/>
+      <c r="C51" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="D51" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" s="10"/>
+      <c r="D51" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="11"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="11" t="s">
+      <c r="A52" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="11"/>
-      <c r="C52" s="11"/>
-      <c r="D52" s="12" t="n">
+      <c r="B52" s="12"/>
+      <c r="C52" s="12"/>
+      <c r="D52" s="13" t="n">
         <f aca="false">SUM(D49:D51)</f>
         <v>4</v>
       </c>
-      <c r="E52" s="13"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="14" t="s">
+      <c r="E52" s="14"/>
+    </row>
+    <row r="53" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B53" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="15" t="n">
-        <f aca="false">D10+D16+D21+D26+D33+D38+D43+D48+D52</f>
+      <c r="C53" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="B54" s="10"/>
+      <c r="C54" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B55" s="10"/>
+      <c r="C55" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" s="8" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="B56" s="10"/>
+      <c r="C56" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" s="11" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B57" s="10"/>
+      <c r="C57" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E57" s="8"/>
+    </row>
+    <row r="58" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="B58" s="10"/>
+      <c r="C58" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D58" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" s="11" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B59" s="10"/>
+      <c r="C59" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E59" s="8"/>
+    </row>
+    <row r="60" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="9" t="n">
         <v>46</v>
       </c>
-      <c r="E54" s="16"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="17" t="str">
-        <f aca="false">"Tương đương " &amp; TEXT(D54/8,"0.0") &amp; " ngày làm việc (8 giờ/ngày)"</f>
-        <v>Tương đương 5.8 ngày làm việc (8 giờ/ngày)</v>
-      </c>
-      <c r="B55" s="17"/>
-      <c r="C55" s="17"/>
-      <c r="D55" s="17"/>
-      <c r="E55" s="17"/>
+      <c r="B60" s="10"/>
+      <c r="C60" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="D60" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E60" s="11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B61" s="10"/>
+      <c r="C61" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E61" s="8"/>
+    </row>
+    <row r="62" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="B62" s="10"/>
+      <c r="C62" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D62" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E62" s="11"/>
+    </row>
+    <row r="63" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B63" s="10"/>
+      <c r="C63" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E63" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="B64" s="12"/>
+      <c r="C64" s="12"/>
+      <c r="D64" s="13" t="n">
+        <f aca="false">SUM(D53:D63)</f>
+        <v>21.5</v>
+      </c>
+      <c r="E64" s="14"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="B66" s="15"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="16" t="n">
+        <f aca="false">D10+D16+D21+D26+D33+D38+D43+D48+D52+D64</f>
+        <v>67.5</v>
+      </c>
+      <c r="E66" s="17"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="18" t="str">
+        <f aca="false">"Tương đương " &amp; TEXT(D66/8,"0.0") &amp; " ngày làm việc (8 giờ/ngày)"</f>
+        <v>Tương đương 8.4 ngày làm việc (8 giờ/ngày)</v>
+      </c>
+      <c r="B67" s="18"/>
+      <c r="C67" s="18"/>
+      <c r="D67" s="18"/>
+      <c r="E67" s="18"/>
+    </row>
+    <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B68" s="19"/>
+      <c r="C68" s="19"/>
+      <c r="D68" s="19"/>
+      <c r="E68" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="26">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
@@ -1508,8 +1759,11 @@
     <mergeCell ref="A48:C48"/>
     <mergeCell ref="B49:B51"/>
     <mergeCell ref="A52:C52"/>
-    <mergeCell ref="A54:C54"/>
-    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="B53:B63"/>
+    <mergeCell ref="A64:C64"/>
+    <mergeCell ref="A66:C66"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A68:E68"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>